<commit_message>
update PDF dan Import
</commit_message>
<xml_diff>
--- a/uploads/Template_Import_Journal.xlsx
+++ b/uploads/Template_Import_Journal.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/def358f71f484966/Documents/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\acv-master\uploads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{6D1CD086-F7B7-4F04-A356-E00C4A849048}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{61157CF6-4FFC-47DC-B08A-834B60AF4143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{F1E41195-A436-4E53-BFEC-2E2372664A99}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="18">
   <si>
     <t>journal_date</t>
   </si>
@@ -84,6 +84,12 @@
   </si>
   <si>
     <t>Description 2</t>
+  </si>
+  <si>
+    <t>status</t>
+  </si>
+  <si>
+    <t>new</t>
   </si>
 </sst>
 </file>
@@ -119,7 +125,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -142,12 +148,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -159,6 +178,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -496,7 +518,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{588D8980-4538-435A-8B4C-FDDA97F3307D}">
-  <dimension ref="A1:H4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.5703125" style="3" customWidth="1"/>
@@ -510,7 +532,7 @@
     <col min="9" max="9" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -535,8 +557,11 @@
       <c r="H1" s="4" t="s">
         <v>7</v>
       </c>
+      <c r="I1" s="5" t="s">
+        <v>16</v>
+      </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>44562</v>
       </c>
@@ -561,8 +586,11 @@
       <c r="H2" s="1">
         <v>50000</v>
       </c>
+      <c r="I2" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>44563</v>
       </c>
@@ -587,8 +615,11 @@
       <c r="H3" s="1">
         <v>150000</v>
       </c>
+      <c r="I3" t="s">
+        <v>17</v>
+      </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
       <c r="B4" s="1"/>
       <c r="C4" s="1"/>

</xml_diff>